<commit_message>
feat(preflight): Phase 3 — 5 new pre-flight validation checks
Added to topology_engine.py validate():
- Check 5: wait_for targets must exist in topology
- Check 5b: fan-in size WARN when wait_for > 5 entries (context overflow risk)
- Check 6: circular wait_for dependency detection via DFS (deadlock prevention)
- Check 7: dialogue_partner must exist in agent_roster.csv when dialogue_rounds > 0

Updated T6_VALIDATE: ORPHAN_NODE now also has wait_for=GHOST_NODE to exercise
check 5 alongside the existing dead-end check.

T6 output (zero API cost):
  ORPHAN_NODE  ERROR  next_node_success  Next node 'NONEXISTENT_TARGET' does not exist
  ORPHAN_NODE  ERROR  wait_for           Wait_For target 'GHOST_NODE' does not exist
</commit_message>
<xml_diff>
--- a/__DATACENTER/T6_VALIDATE/MACCRE_Swarm_Request.xlsx
+++ b/__DATACENTER/T6_VALIDATE/MACCRE_Swarm_Request.xlsx
@@ -1368,7 +1368,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Orphan node — unreachable. Routes to a nonexistent target.</t>
+          <t>Orphan node — unreachable. Routes to a nonexistent target. Also waits for a ghost node.</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr"/>
@@ -1387,7 +1387,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>GHOST_NODE</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">

</xml_diff>